<commit_message>
Build historical analysis and WACC assumptions
Updated the valuation model with historical financial analysis and WACC assumptions, including revenue growth, EBITDA, EBIT, tax rate, capex, change in NWC, cost of equity, cost of debt, capital structure weights and terminal growth.
</commit_message>
<xml_diff>
--- a/Pidilite_Stock_Valuation_Model.xlsx
+++ b/Pidilite_Stock_Valuation_Model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\stock valuatioin model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19167508-6D36-475B-A7F7-9DC43841E1C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC1E965-E9C5-4C63-BB38-928114C4B7A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{66F55DBC-AC4A-4A3B-94F5-72EBBB4B874A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
   <si>
     <t>Particulars</t>
   </si>
@@ -141,14 +141,48 @@
   </si>
   <si>
     <t>Terminal Growth</t>
+  </si>
+  <si>
+    <t>Working Capital</t>
+  </si>
+  <si>
+    <t>Risk Free Rate</t>
+  </si>
+  <si>
+    <t>Beta</t>
+  </si>
+  <si>
+    <t>Market Return</t>
+  </si>
+  <si>
+    <t>Cost of Equity</t>
+  </si>
+  <si>
+    <t>Cost of Debt</t>
+  </si>
+  <si>
+    <t>Debt %</t>
+  </si>
+  <si>
+    <t>Equity %</t>
+  </si>
+  <si>
+    <t>Market Cap</t>
+  </si>
+  <si>
+    <t>Debt</t>
+  </si>
+  <si>
+    <t>Total Capital</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="167" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="174" formatCode="0.0000%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -173,7 +207,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -190,6 +224,18 @@
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -209,16 +255,22 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="60% - Accent1 2" xfId="3" xr:uid="{B8273F70-2B0D-4190-A0A8-1142ECEF9ED2}"/>
@@ -537,62 +589,168 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A02ED063-43CB-48D4-A5CA-8CACBDF50116}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="12" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="11">
         <f>AVERAGE(Historicals!C3:F3)</f>
         <v>0.1027756094442282</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="11">
         <f>AVERAGE(Historicals!B5:F5)</f>
         <v>0.20889009323488397</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="11">
         <f>AVERAGE(Historicals!B10:F10)</f>
         <v>0.25662000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="6" t="s">
         <v>30</v>
       </c>
+      <c r="B5">
+        <f>AVERAGE(3.25%,3.64%,4.07%,3.26%,3.92%)</f>
+        <v>3.628E-2</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="6" t="s">
         <v>31</v>
       </c>
+      <c r="B6" s="11">
+        <f>AVERAGE(Historicals!B15:F15)</f>
+        <v>4.7453057351992661E-3</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="6" t="s">
         <v>32</v>
       </c>
+      <c r="B7" s="11">
+        <f>B16*B13+B15*B14*(1-B4)</f>
+        <v>9.7485720303274723E-2</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="6" t="s">
         <v>33</v>
+      </c>
+      <c r="B8" s="14">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="13"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="11">
+        <v>7.1300000000000002E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="11">
+        <v>0.1368</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="4">
+        <f>B10+B11*(B12-B10)</f>
+        <v>9.7500000000000003E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="11">
+        <f>54.22/AVERAGE(454.14,417.21)</f>
+        <v>0.12445056521489643</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="11">
+        <f>B19/B20</f>
+        <v>2.8639935648183709E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16">
+        <f>B18/B20</f>
+        <v>0.99713600643518163</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18">
+        <v>145257</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19">
+        <v>417.21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20">
+        <f>B18+B19</f>
+        <v>145674.21</v>
       </c>
     </row>
   </sheetData>
@@ -602,10 +760,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A029249C-9FB7-4F3D-AEE2-382FA44E25DE}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -632,19 +791,19 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>9920.9599999999991</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>11799.1</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>12382.99</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <v>13140.31</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="2">
         <v>14600.83</v>
       </c>
     </row>
@@ -718,19 +877,19 @@
       <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="7">
         <v>239.61</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="7">
         <v>269.74</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="7">
         <v>340.66</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="7">
         <v>358.48</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="7">
         <v>394.71</v>
       </c>
     </row>
@@ -742,19 +901,19 @@
         <f>B4-B6</f>
         <v>1616.8000000000002</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="7">
         <f t="shared" ref="C7:F7" si="2">C4-C6</f>
         <v>1716.35</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="7">
         <f t="shared" si="2"/>
         <v>2367.79</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="7">
         <f t="shared" si="2"/>
         <v>2652.1</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="7">
         <f t="shared" si="2"/>
         <v>3126.59</v>
       </c>
@@ -763,23 +922,23 @@
       <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="8">
         <f>B7/B2</f>
         <v>0.16296809986130378</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="8">
         <f t="shared" ref="C8:F8" si="3">C7/C2</f>
         <v>0.14546448457933231</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="8">
         <f t="shared" si="3"/>
         <v>0.19121310765816657</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="8">
         <f t="shared" si="3"/>
         <v>0.20182933279351858</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="8">
         <f t="shared" si="3"/>
         <v>0.21413782641123827</v>
       </c>
@@ -788,19 +947,19 @@
       <c r="A9" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="9">
         <v>407.02</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="9">
         <v>434.37</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="9">
         <v>631.92999999999995</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="9">
         <v>726.53</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="9">
         <v>849.45</v>
       </c>
     </row>
@@ -828,19 +987,19 @@
       <c r="A11" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="10">
         <v>1207.56</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="10">
         <v>1273.25</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="10">
         <v>1729.38</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="10">
         <v>2076.2399999999998</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="10">
         <v>2448.92</v>
       </c>
     </row>
@@ -848,25 +1007,94 @@
       <c r="A12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="11">
         <f>B11/B2</f>
         <v>0.12171805954262491</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="11">
         <f t="shared" ref="C12:F12" si="4">C11/C2</f>
         <v>0.10791077285555678</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="11">
         <f t="shared" si="4"/>
         <v>0.13965770787184678</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="11">
         <f t="shared" si="4"/>
         <v>0.15800540474311489</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="11">
         <f t="shared" si="4"/>
         <v>0.16772471154037133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13">
+        <v>1432.25</v>
+      </c>
+      <c r="C13">
+        <v>1402.02</v>
+      </c>
+      <c r="D13">
+        <v>955.87</v>
+      </c>
+      <c r="E13">
+        <v>823.04</v>
+      </c>
+      <c r="F13">
+        <v>797.27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="3">
+        <v>736.05</v>
+      </c>
+      <c r="C14">
+        <f>C13-B13</f>
+        <v>-30.230000000000018</v>
+      </c>
+      <c r="D14" s="10">
+        <f t="shared" ref="D14:F14" si="5">D13-C13</f>
+        <v>-446.15</v>
+      </c>
+      <c r="E14" s="10">
+        <f t="shared" si="5"/>
+        <v>-132.83000000000004</v>
+      </c>
+      <c r="F14" s="10">
+        <f t="shared" si="5"/>
+        <v>-25.769999999999982</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="1">
+        <f>B14/B2</f>
+        <v>7.4191408895913302E-2</v>
+      </c>
+      <c r="C15" s="1">
+        <f t="shared" ref="C15:F15" si="6">C14/C2</f>
+        <v>-2.5620598181217225E-3</v>
+      </c>
+      <c r="D15" s="1">
+        <f t="shared" si="6"/>
+        <v>-3.6029262722492711E-2</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="6"/>
+        <v>-1.0108589523382634E-2</v>
+      </c>
+      <c r="F15" s="1">
+        <f t="shared" si="6"/>
+        <v>-1.764968155919902E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update valuation model through DCF sensitivity analysis
</commit_message>
<xml_diff>
--- a/Pidilite_Stock_Valuation_Model.xlsx
+++ b/Pidilite_Stock_Valuation_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\stock valuatioin model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC1E965-E9C5-4C63-BB38-928114C4B7A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA310B1-3BE8-438A-B51A-CD9989AE3C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{66F55DBC-AC4A-4A3B-94F5-72EBBB4B874A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="2" xr2:uid="{66F55DBC-AC4A-4A3B-94F5-72EBBB4B874A}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -38,8 +38,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="68">
   <si>
     <t>Particulars</t>
   </si>
@@ -174,6 +196,75 @@
   </si>
   <si>
     <t>Total Capital</t>
+  </si>
+  <si>
+    <t>D&amp;A % of Revenue</t>
+  </si>
+  <si>
+    <t>Discount Factor</t>
+  </si>
+  <si>
+    <t>Present Value of FCFF</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>PV of Forecast FCFF</t>
+  </si>
+  <si>
+    <t>Terminal Value</t>
+  </si>
+  <si>
+    <t>PV of Terminal Value</t>
+  </si>
+  <si>
+    <t>Enterprise Value</t>
+  </si>
+  <si>
+    <t>Net Debt</t>
+  </si>
+  <si>
+    <t>Equity Value</t>
+  </si>
+  <si>
+    <t>Shares Outstanding (Cr)</t>
+  </si>
+  <si>
+    <t>Cash &amp; Bank (₹ Cr)</t>
+  </si>
+  <si>
+    <t>Note: Monetary values are in ₹ Crore unless otherwise stated.</t>
+  </si>
+  <si>
+    <t>DCF Valuation (₹ Cr, except per-share value)</t>
+  </si>
+  <si>
+    <t>Comparable Company Valuation (₹ Cr, except per-share data &amp; multiples)</t>
+  </si>
+  <si>
+    <t>Valuation Summary (₹ Cr, except per-share data)</t>
+  </si>
+  <si>
+    <t>Note: Monetary values are in ₹ Crore; percentages are shown as %.</t>
+  </si>
+  <si>
+    <t>Current Market Price (₹)</t>
+  </si>
+  <si>
+    <t>Upside / (Downside) %</t>
+  </si>
+  <si>
+    <t>Valuation Date</t>
+  </si>
+  <si>
+    <t>Intrinsic Value / Share (₹)</t>
+  </si>
+  <si>
+    <t>Sensitivity Analysis — Intrinsic Value / Share (₹)</t>
+  </si>
+  <si>
+    <t>WACC \ Terminal Growth</t>
   </si>
 </sst>
 </file>
@@ -184,7 +275,7 @@
     <numFmt numFmtId="167" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="174" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -195,6 +286,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -252,10 +350,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -269,8 +367,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="60% - Accent1 2" xfId="3" xr:uid="{B8273F70-2B0D-4190-A0A8-1142ECEF9ED2}"/>
@@ -589,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A02ED063-43CB-48D4-A5CA-8CACBDF50116}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
@@ -634,7 +734,7 @@
       <c r="A5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="11">
         <f>AVERAGE(3.25%,3.64%,4.07%,3.26%,3.92%)</f>
         <v>3.628E-2</v>
       </c>
@@ -661,12 +761,18 @@
       <c r="A8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="13">
         <v>0.05</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="13"/>
+      <c r="A9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="1">
+        <f>AVERAGE(Historicals!B6/Historicals!B2,Historicals!C6/Historicals!C2,Historicals!D6/Historicals!D2,Historicals!E6/Historicals!E2,Historicals!F6/Historicals!F2)</f>
+        <v>2.5767522974172084E-2</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
@@ -723,7 +829,7 @@
       <c r="A16" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="11">
         <f>B18/B20</f>
         <v>0.99713600643518163</v>
       </c>
@@ -753,14 +859,36 @@
         <v>145674.21</v>
       </c>
     </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21">
+        <v>298.89999999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22">
+        <v>101.7766</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="14" t="s">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A029249C-9FB7-4F3D-AEE2-382FA44E25DE}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.54296875" customWidth="1"/>
@@ -1097,15 +1225,24 @@
         <v>-1.764968155919902E-3</v>
       </c>
     </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="14" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2095F5-79CA-42C2-80D9-9AE2D355E225}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1131,60 +1268,305 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
+      <c r="B2">
+        <f>Historicals!F2*(1+B3)</f>
+        <v>16101.439201641571</v>
+      </c>
+      <c r="C2" s="10">
+        <f>B2*(1+C3)</f>
+        <v>17756.274428519471</v>
+      </c>
+      <c r="D2" s="10">
+        <f t="shared" ref="D2:F2" si="0">C2*(1+D3)</f>
+        <v>19581.186354369525</v>
+      </c>
+      <c r="E2" s="10">
+        <f t="shared" si="0"/>
+        <v>21593.654715580858</v>
+      </c>
+      <c r="F2" s="10">
+        <f t="shared" si="0"/>
+        <v>23812.955739102916</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
+      <c r="B3" s="11">
+        <f>Inputs!$B$2</f>
+        <v>0.1027756094442282</v>
+      </c>
+      <c r="C3" s="11">
+        <f>Inputs!$B$2</f>
+        <v>0.1027756094442282</v>
+      </c>
+      <c r="D3" s="11">
+        <f>Inputs!$B$2</f>
+        <v>0.1027756094442282</v>
+      </c>
+      <c r="E3" s="11">
+        <f>Inputs!$B$2</f>
+        <v>0.1027756094442282</v>
+      </c>
+      <c r="F3" s="11">
+        <f>Inputs!$B$2</f>
+        <v>0.1027756094442282</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
+      <c r="B4">
+        <f>B2*B5</f>
+        <v>3363.4311360467236</v>
+      </c>
+      <c r="C4" s="10">
+        <f t="shared" ref="C4:F4" si="1">C2*C5</f>
+        <v>3709.1098208776184</v>
+      </c>
+      <c r="D4" s="10">
+        <f t="shared" si="1"/>
+        <v>4090.315843213888</v>
+      </c>
+      <c r="E4" s="10">
+        <f t="shared" si="1"/>
+        <v>4510.7005468195775</v>
+      </c>
+      <c r="F4" s="10">
+        <f t="shared" si="1"/>
+        <v>4974.2905445393735</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
+      <c r="B5" s="11">
+        <f>Inputs!$B$3</f>
+        <v>0.20889009323488397</v>
+      </c>
+      <c r="C5" s="11">
+        <f>Inputs!$B$3</f>
+        <v>0.20889009323488397</v>
+      </c>
+      <c r="D5" s="11">
+        <f>Inputs!$B$3</f>
+        <v>0.20889009323488397</v>
+      </c>
+      <c r="E5" s="11">
+        <f>Inputs!$B$3</f>
+        <v>0.20889009323488397</v>
+      </c>
+      <c r="F5" s="11">
+        <f>Inputs!$B$3</f>
+        <v>0.20889009323488397</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
+      <c r="B6" s="3">
+        <f>B2*Inputs!$B$9</f>
+        <v>414.89420454553419</v>
+      </c>
+      <c r="C6" s="3">
+        <f>C2*Inputs!$B$9</f>
+        <v>457.53520927257978</v>
+      </c>
+      <c r="D6" s="3">
+        <f>D2*Inputs!$B$9</f>
+        <v>504.55866924776166</v>
+      </c>
+      <c r="E6" s="3">
+        <f>E2*Inputs!$B$9</f>
+        <v>556.41499398006908</v>
+      </c>
+      <c r="F6" s="3">
+        <f>F2*Inputs!$B$9</f>
+        <v>613.60088409027742</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
+      <c r="B7">
+        <f>B4-B6</f>
+        <v>2948.5369315011894</v>
+      </c>
+      <c r="C7" s="10">
+        <f t="shared" ref="C7:F7" si="2">C4-C6</f>
+        <v>3251.5746116050386</v>
+      </c>
+      <c r="D7" s="10">
+        <f t="shared" si="2"/>
+        <v>3585.7571739661262</v>
+      </c>
+      <c r="E7" s="10">
+        <f t="shared" si="2"/>
+        <v>3954.2855528395085</v>
+      </c>
+      <c r="F7" s="10">
+        <f t="shared" si="2"/>
+        <v>4360.6896604490958</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
+      <c r="B8" s="11">
+        <f>Inputs!$B$4</f>
+        <v>0.25662000000000001</v>
+      </c>
+      <c r="C8" s="11">
+        <f>Inputs!$B$4</f>
+        <v>0.25662000000000001</v>
+      </c>
+      <c r="D8" s="11">
+        <f>Inputs!$B$4</f>
+        <v>0.25662000000000001</v>
+      </c>
+      <c r="E8" s="11">
+        <f>Inputs!$B$4</f>
+        <v>0.25662000000000001</v>
+      </c>
+      <c r="F8" s="11">
+        <f>Inputs!$B$4</f>
+        <v>0.25662000000000001</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
+      <c r="B9">
+        <f>B7*B8</f>
+        <v>756.65354736183531</v>
+      </c>
+      <c r="C9" s="10">
+        <f t="shared" ref="C9:F9" si="3">C7*C8</f>
+        <v>834.41907683008503</v>
+      </c>
+      <c r="D9" s="10">
+        <f t="shared" si="3"/>
+        <v>920.17700598318731</v>
+      </c>
+      <c r="E9" s="10">
+        <f t="shared" si="3"/>
+        <v>1014.7487585696747</v>
+      </c>
+      <c r="F9" s="10">
+        <f t="shared" si="3"/>
+        <v>1119.040180664447</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
+      <c r="B10">
+        <f>B7*(1-B8)</f>
+        <v>2191.8833841393539</v>
+      </c>
+      <c r="C10" s="10">
+        <f t="shared" ref="C10:F10" si="4">C7*(1-C8)</f>
+        <v>2417.1555347749536</v>
+      </c>
+      <c r="D10" s="10">
+        <f t="shared" si="4"/>
+        <v>2665.5801679829387</v>
+      </c>
+      <c r="E10" s="10">
+        <f t="shared" si="4"/>
+        <v>2939.5367942698335</v>
+      </c>
+      <c r="F10" s="10">
+        <f t="shared" si="4"/>
+        <v>3241.6494797846485</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>23</v>
       </c>
+      <c r="B11" s="10">
+        <f>B2*Inputs!$B$5</f>
+        <v>584.16021423555617</v>
+      </c>
+      <c r="C11" s="10">
+        <f>C2*Inputs!$B$5</f>
+        <v>644.19763626668646</v>
+      </c>
+      <c r="D11" s="10">
+        <f>D2*Inputs!$B$5</f>
+        <v>710.40544093652636</v>
+      </c>
+      <c r="E11" s="10">
+        <f>E2*Inputs!$B$5</f>
+        <v>783.41779308127354</v>
+      </c>
+      <c r="F11" s="10">
+        <f>F2*Inputs!$B$5</f>
+        <v>863.93403421465382</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>24</v>
       </c>
+      <c r="B12" s="10">
+        <f>B2*Inputs!$B$6</f>
+        <v>76.406251788512037</v>
+      </c>
+      <c r="C12" s="10">
+        <f>C2*Inputs!$B$6</f>
+        <v>84.25895088142552</v>
+      </c>
+      <c r="D12" s="10">
+        <f>D2*Inputs!$B$6</f>
+        <v>92.918715909395317</v>
+      </c>
+      <c r="E12" s="10">
+        <f>E2*Inputs!$B$6</f>
+        <v>102.46849356575852</v>
+      </c>
+      <c r="F12" s="10">
+        <f>F2*Inputs!$B$6</f>
+        <v>112.99975544081134</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
+      </c>
+      <c r="B13" s="10">
+        <f>B10+B6-B11-B12</f>
+        <v>1946.2111226608199</v>
+      </c>
+      <c r="C13" s="10">
+        <f t="shared" ref="C13:F13" si="5">C10+C6-C11-C12</f>
+        <v>2146.2341568994216</v>
+      </c>
+      <c r="D13" s="10">
+        <f t="shared" si="5"/>
+        <v>2366.814680384779</v>
+      </c>
+      <c r="E13" s="10">
+        <f t="shared" si="5"/>
+        <v>2610.0655016028709</v>
+      </c>
+      <c r="F13" s="10">
+        <f t="shared" si="5"/>
+        <v>2878.3165742194606</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="14" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1194,10 +1576,405 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4A60EBC-8083-4456-B121-9DB07E3866D2}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="9.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4">
+        <f>Forecast!B13</f>
+        <v>1946.2111226608199</v>
+      </c>
+      <c r="C4" s="10">
+        <f>Forecast!C13</f>
+        <v>2146.2341568994216</v>
+      </c>
+      <c r="D4" s="10">
+        <f>Forecast!D13</f>
+        <v>2366.814680384779</v>
+      </c>
+      <c r="E4" s="10">
+        <f>Forecast!E13</f>
+        <v>2610.0655016028709</v>
+      </c>
+      <c r="F4" s="10">
+        <f>Forecast!F13</f>
+        <v>2878.3165742194606</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5">
+        <f>1/(1+$B$8)^B11</f>
+        <v>0.91117358658995962</v>
+      </c>
+      <c r="C5" s="10">
+        <f t="shared" ref="C5:F5" si="0">1/(1+$B$8)^C11</f>
+        <v>0.83023730489921055</v>
+      </c>
+      <c r="D5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.75649030282579555</v>
+      </c>
+      <c r="E5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.68929398244630469</v>
+      </c>
+      <c r="F5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.62806647020047612</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6">
+        <f>B4*B5</f>
+        <v>1773.3361688961311</v>
+      </c>
+      <c r="C6" s="10">
+        <f t="shared" ref="C6:F6" si="1">C4*C5</f>
+        <v>1781.8836621068051</v>
+      </c>
+      <c r="D6" s="10">
+        <f t="shared" si="1"/>
+        <v>1790.47235429682</v>
+      </c>
+      <c r="E6" s="10">
+        <f t="shared" si="1"/>
+        <v>1799.1024440455546</v>
+      </c>
+      <c r="F6" s="10">
+        <f t="shared" si="1"/>
+        <v>1807.7741308895434</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="11">
+        <f>Inputs!B7</f>
+        <v>9.7485720303274723E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="13">
+        <f>Inputs!B8</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" s="10">
+        <v>2</v>
+      </c>
+      <c r="D11" s="10">
+        <v>3</v>
+      </c>
+      <c r="E11" s="10">
+        <v>4</v>
+      </c>
+      <c r="F11" s="10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12">
+        <f>SUM(B6:F6)</f>
+        <v>8952.5687602348553</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14">
+        <f>F4*(1+$B$9)/($B$8-$B$9)</f>
+        <v>63645.078638977997</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15">
+        <f>B14*F5</f>
+        <v>39973.339886414637</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16">
+        <f>B12+B15</f>
+        <v>48925.908646649492</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17">
+        <f>Inputs!B19-Inputs!B21</f>
+        <v>118.31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18">
+        <f>B16-B17</f>
+        <v>48807.598646649494</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19">
+        <f>Inputs!B22</f>
+        <v>101.7766</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20">
+        <f>B18/B19</f>
+        <v>479.55619117409594</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22">
+        <v>1517.2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="1">
+        <f>(B20/B22)-1</f>
+        <v>-0.68392025364217246</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="15">
+        <f>DATE(2026,9,25)</f>
+        <v>46290</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>67</v>
+      </c>
+      <c r="B28" s="13">
+        <v>0.04</v>
+      </c>
+      <c r="C28" s="11">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="D28" s="13">
+        <f>$B$9</f>
+        <v>0.05</v>
+      </c>
+      <c r="E28" s="11">
+        <v>5.5E-2</v>
+      </c>
+      <c r="F28" s="13">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="1">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="B29" s="16" cm="1">
+        <f t="array" ref="B29">(SUMPRODUCT($B$4:$F$4/(1+$A29)^$B$11:$F$11)+($F$4*(1+B$28)/( $A29-B$28))/(1+$A29)^$F$11-$B$17)/$B$19</f>
+        <v>496.34539643750281</v>
+      </c>
+      <c r="C29" s="16" cm="1">
+        <f t="array" ref="C29">(SUMPRODUCT($B$4:$F$4/(1+$A29)^$B$11:$F$11)+($F$4*(1+C$28)/( $A29-C$28))/(1+$A29)^$F$11-$B$17)/$B$19</f>
+        <v>546.42501612649482</v>
+      </c>
+      <c r="D29" s="16" cm="1">
+        <f t="array" ref="D29">(SUMPRODUCT($B$4:$F$4/(1+$A29)^$B$11:$F$11)+($F$4*(1+D$28)/( $A29-D$28))/(1+$A29)^$F$11-$B$17)/$B$19</f>
+        <v>609.85920106588503</v>
+      </c>
+      <c r="E29" s="16" cm="1">
+        <f t="array" ref="E29">(SUMPRODUCT($B$4:$F$4/(1+$A29)^$B$11:$F$11)+($F$4*(1+E$28)/( $A29-E$28))/(1+$A29)^$F$11-$B$17)/$B$19</f>
+        <v>692.8115967558565</v>
+      </c>
+      <c r="F29" s="16" cm="1">
+        <f t="array" ref="F29">(SUMPRODUCT($B$4:$F$4/(1+$A29)^$B$11:$F$11)+($F$4*(1+F$28)/( $A29-F$28))/(1+$A29)^$F$11-$B$17)/$B$19</f>
+        <v>805.92849996945404</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="1">
+        <v>9.2499999999999999E-2</v>
+      </c>
+      <c r="B30" s="16" cm="1">
+        <f t="array" ref="B30">(SUMPRODUCT($B$4:$F$4/(1+$A30)^$B$11:$F$11)+($F$4*(1+B$28)/( $A30-B$28))/(1+$A30)^$F$11-$B$17)/$B$19</f>
+        <v>447.97866707565385</v>
+      </c>
+      <c r="C30" s="16" cm="1">
+        <f t="array" ref="C30">(SUMPRODUCT($B$4:$F$4/(1+$A30)^$B$11:$F$11)+($F$4*(1+C$28)/( $A30-C$28))/(1+$A30)^$F$11-$B$17)/$B$19</f>
+        <v>487.78222816914212</v>
+      </c>
+      <c r="D30" s="16" cm="1">
+        <f t="array" ref="D30">(SUMPRODUCT($B$4:$F$4/(1+$A30)^$B$11:$F$11)+($F$4*(1+D$28)/( $A30-D$28))/(1+$A30)^$F$11-$B$17)/$B$19</f>
+        <v>536.95133304933347</v>
+      </c>
+      <c r="E30" s="16" cm="1">
+        <f t="array" ref="E30">(SUMPRODUCT($B$4:$F$4/(1+$A30)^$B$11:$F$11)+($F$4*(1+E$28)/( $A30-E$28))/(1+$A30)^$F$11-$B$17)/$B$19</f>
+        <v>599.23219923090926</v>
+      </c>
+      <c r="F30" s="16" cm="1">
+        <f t="array" ref="F30">(SUMPRODUCT($B$4:$F$4/(1+$A30)^$B$11:$F$11)+($F$4*(1+F$28)/( $A30-F$28))/(1+$A30)^$F$11-$B$17)/$B$19</f>
+        <v>680.67640885296998</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
+        <f>$B$8</f>
+        <v>9.7485720303274723E-2</v>
+      </c>
+      <c r="B31" s="16" cm="1">
+        <f t="array" ref="B31">(SUMPRODUCT($B$4:$F$4/(1+$A31)^$B$11:$F$11)+($F$4*(1+B$28)/( $A31-B$28))/(1+$A31)^$F$11-$B$17)/$B$19</f>
+        <v>408.14404266840728</v>
+      </c>
+      <c r="C31" s="16" cm="1">
+        <f t="array" ref="C31">(SUMPRODUCT($B$4:$F$4/(1+$A31)^$B$11:$F$11)+($F$4*(1+C$28)/( $A31-C$28))/(1+$A31)^$F$11-$B$17)/$B$19</f>
+        <v>440.44861323162638</v>
+      </c>
+      <c r="D31" s="16" cm="1">
+        <f t="array" ref="D31">(SUMPRODUCT($B$4:$F$4/(1+$A31)^$B$11:$F$11)+($F$4*(1+D$28)/( $A31-D$28))/(1+$A31)^$F$11-$B$17)/$B$19</f>
+        <v>479.55619117409594</v>
+      </c>
+      <c r="E31" s="16" cm="1">
+        <f t="array" ref="E31">(SUMPRODUCT($B$4:$F$4/(1+$A31)^$B$11:$F$11)+($F$4*(1+E$28)/( $A31-E$28))/(1+$A31)^$F$11-$B$17)/$B$19</f>
+        <v>527.86864493444216</v>
+      </c>
+      <c r="F31" s="16" cm="1">
+        <f t="array" ref="F31">(SUMPRODUCT($B$4:$F$4/(1+$A31)^$B$11:$F$11)+($F$4*(1+F$28)/( $A31-F$28))/(1+$A31)^$F$11-$B$17)/$B$19</f>
+        <v>589.06932743081893</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="1">
+        <v>0.10249999999999999</v>
+      </c>
+      <c r="B32" s="16" cm="1">
+        <f t="array" ref="B32">(SUMPRODUCT($B$4:$F$4/(1+$A32)^$B$11:$F$11)+($F$4*(1+B$28)/( $A32-B$28))/(1+$A32)^$F$11-$B$17)/$B$19</f>
+        <v>374.50601510905022</v>
+      </c>
+      <c r="C32" s="16" cm="1">
+        <f t="array" ref="C32">(SUMPRODUCT($B$4:$F$4/(1+$A32)^$B$11:$F$11)+($F$4*(1+C$28)/( $A32-C$28))/(1+$A32)^$F$11-$B$17)/$B$19</f>
+        <v>401.13768320750921</v>
+      </c>
+      <c r="D32" s="16" cm="1">
+        <f t="array" ref="D32">(SUMPRODUCT($B$4:$F$4/(1+$A32)^$B$11:$F$11)+($F$4*(1+D$28)/( $A32-D$28))/(1+$A32)^$F$11-$B$17)/$B$19</f>
+        <v>432.84204999138916</v>
+      </c>
+      <c r="E32" s="16" cm="1">
+        <f t="array" ref="E32">(SUMPRODUCT($B$4:$F$4/(1+$A32)^$B$11:$F$11)+($F$4*(1+E$28)/( $A32-E$28))/(1+$A32)^$F$11-$B$17)/$B$19</f>
+        <v>471.2210203087173</v>
+      </c>
+      <c r="F32" s="16" cm="1">
+        <f t="array" ref="F32">(SUMPRODUCT($B$4:$F$4/(1+$A32)^$B$11:$F$11)+($F$4*(1+F$28)/( $A32-F$28))/(1+$A32)^$F$11-$B$17)/$B$19</f>
+        <v>518.63033658306404</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="1">
+        <v>0.1075</v>
+      </c>
+      <c r="B33" s="16" cm="1">
+        <f t="array" ref="B33">(SUMPRODUCT($B$4:$F$4/(1+$A33)^$B$11:$F$11)+($F$4*(1+B$28)/( $A33-B$28))/(1+$A33)^$F$11-$B$17)/$B$19</f>
+        <v>345.95339591019837</v>
+      </c>
+      <c r="C33" s="16" cm="1">
+        <f t="array" ref="C33">(SUMPRODUCT($B$4:$F$4/(1+$A33)^$B$11:$F$11)+($F$4*(1+C$28)/( $A33-C$28))/(1+$A33)^$F$11-$B$17)/$B$19</f>
+        <v>368.23271402248685</v>
+      </c>
+      <c r="D33" s="16" cm="1">
+        <f t="array" ref="D33">(SUMPRODUCT($B$4:$F$4/(1+$A33)^$B$11:$F$11)+($F$4*(1+D$28)/( $A33-D$28))/(1+$A33)^$F$11-$B$17)/$B$19</f>
+        <v>394.38669615430388</v>
+      </c>
+      <c r="E33" s="16" cm="1">
+        <f t="array" ref="E33">(SUMPRODUCT($B$4:$F$4/(1+$A33)^$B$11:$F$11)+($F$4*(1+E$28)/( $A33-E$28))/(1+$A33)^$F$11-$B$17)/$B$19</f>
+        <v>425.5223891683716</v>
+      </c>
+      <c r="F33" s="16" cm="1">
+        <f t="array" ref="F33">(SUMPRODUCT($B$4:$F$4/(1+$A33)^$B$11:$F$11)+($F$4*(1+F$28)/( $A33-F$28))/(1+$A33)^$F$11-$B$17)/$B$19</f>
+        <v>463.2129649222432</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1205,7 +1982,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B394838-33E4-44C6-B04A-2645A3556A9B}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1214,7 +1997,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8FB6CAA-755E-4048-8F46-C387A89B309E}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Pidilite valuation model
</commit_message>
<xml_diff>
--- a/Pidilite_Stock_Valuation_Model.xlsx
+++ b/Pidilite_Stock_Valuation_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\stock valuatioin model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA310B1-3BE8-438A-B51A-CD9989AE3C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11991639-753C-418C-AD56-68C546E909EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="2" xr2:uid="{66F55DBC-AC4A-4A3B-94F5-72EBBB4B874A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="5" xr2:uid="{66F55DBC-AC4A-4A3B-94F5-72EBBB4B874A}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="103">
   <si>
     <t>Particulars</t>
   </si>
@@ -265,6 +265,111 @@
   </si>
   <si>
     <t>WACC \ Terminal Growth</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>P/E</t>
+  </si>
+  <si>
+    <t>EV/EBITDA</t>
+  </si>
+  <si>
+    <t>Market Cap (₹ Cr)</t>
+  </si>
+  <si>
+    <t>Enterprise Value (₹ Cr)</t>
+  </si>
+  <si>
+    <t>Data Date</t>
+  </si>
+  <si>
+    <t>Nikhil Adhesives</t>
+  </si>
+  <si>
+    <t>HP Adhesives</t>
+  </si>
+  <si>
+    <t>Jyoti Resins</t>
+  </si>
+  <si>
+    <t>Hindustan Adhesive</t>
+  </si>
+  <si>
+    <t>Peer Median</t>
+  </si>
+  <si>
+    <t>Pidilite Implied Valuation</t>
+  </si>
+  <si>
+    <t>P/E Method</t>
+  </si>
+  <si>
+    <t>Implied Equity Value (₹ Cr)</t>
+  </si>
+  <si>
+    <t>Implied Value / Share (₹)</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>EV/EBITDA Method</t>
+  </si>
+  <si>
+    <t>Valuation Method</t>
+  </si>
+  <si>
+    <t>DCF</t>
+  </si>
+  <si>
+    <t>DCF Sensitivity — Low</t>
+  </si>
+  <si>
+    <t>DCF Sensitivity — High</t>
+  </si>
+  <si>
+    <t>P/E Comps</t>
+  </si>
+  <si>
+    <t>EV/EBITDA Comps</t>
+  </si>
+  <si>
+    <t>Current Market Price</t>
+  </si>
+  <si>
+    <t>Key Assumption</t>
+  </si>
+  <si>
+    <t>DCF Valuation Detail</t>
+  </si>
+  <si>
+    <t>Net Debt (₹ Cr)</t>
+  </si>
+  <si>
+    <t>Equity Value (₹ Cr)</t>
+  </si>
+  <si>
+    <t>Comparable Valuation</t>
+  </si>
+  <si>
+    <t>Median Multiple</t>
+  </si>
+  <si>
+    <t>Low (₹)</t>
+  </si>
+  <si>
+    <t>High (₹)</t>
+  </si>
+  <si>
+    <t>DCF Sensitivity</t>
+  </si>
+  <si>
+    <t>DCF Base Case</t>
+  </si>
+  <si>
+    <t>Range (₹)</t>
   </si>
 </sst>
 </file>
@@ -353,7 +458,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -371,6 +476,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="60% - Accent1 2" xfId="3" xr:uid="{B8273F70-2B0D-4190-A0A8-1142ECEF9ED2}"/>
@@ -381,6 +487,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF0B1220"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -390,6 +501,1169 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>Pidilite Industries — Valuation Range (₹ / Share)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Output!$F$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Low (₹)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="inBase"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Output!$E$4:$E$8</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>DCF Sensitivity</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>DCF Base Case</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>P/E Comps</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>EV/EBITDA Comps</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Current Market Price</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Output!$F$4:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0" formatCode="0.00">
+                  <c:v>345.95339591019837</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>479.55619117409594</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>431.18601328792676</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>336.3442235248574</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1517.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A1FC-455D-8EA6-4A3641C61DBE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Output!$H$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Range (₹)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Output!$E$4:$E$8</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>DCF Sensitivity</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>DCF Base Case</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>P/E Comps</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>EV/EBITDA Comps</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Current Market Price</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Output!$H$4:$H$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0" formatCode="0.00">
+                  <c:v>459.97510405925567</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-A1FC-455D-8EA6-4A3641C61DBE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="765543984"/>
+        <c:axId val="571504880"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Output!$G$3</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>High (₹)</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:solidFill>
+                    <a:schemeClr val="accent2"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Output!$E$4:$E$8</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="5"/>
+                      <c:pt idx="0">
+                        <c:v>DCF Sensitivity</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>DCF Base Case</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>P/E Comps</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>EV/EBITDA Comps</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>Current Market Price</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Output!$G$4:$G$8</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="5"/>
+                      <c:pt idx="0" formatCode="0.00">
+                        <c:v>805.92849996945404</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>479.55619117409594</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>431.18601328792676</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>336.3442235248574</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>1517.2</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-A1FC-455D-8EA6-4A3641C61DBE}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+          </c:ext>
+        </c:extLst>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="765543984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="571504880"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="571504880"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765543984"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3175</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>307975</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>174625</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0ADCD0C0-C0BA-43FA-8877-8FD153B60A5A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1980,12 +3254,170 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B394838-33E4-44C6-B04A-2645A3556A9B}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="6" max="6" width="9.08984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4">
+        <v>12.07</v>
+      </c>
+      <c r="C4">
+        <v>7.51</v>
+      </c>
+      <c r="D4">
+        <v>844.44</v>
+      </c>
+      <c r="E4">
+        <v>638.35</v>
+      </c>
+      <c r="F4" s="17">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5">
+        <v>23.77</v>
+      </c>
+      <c r="C5">
+        <v>12</v>
+      </c>
+      <c r="D5">
+        <v>400.73</v>
+      </c>
+      <c r="E5">
+        <v>444.6</v>
+      </c>
+      <c r="F5" s="17">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6">
+        <v>24.37</v>
+      </c>
+      <c r="C6">
+        <v>14.49</v>
+      </c>
+      <c r="D6">
+        <v>442.27</v>
+      </c>
+      <c r="E6">
+        <v>370.07</v>
+      </c>
+      <c r="F6" s="17">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7">
+        <v>11.19</v>
+      </c>
+      <c r="C7">
+        <v>7.01</v>
+      </c>
+      <c r="D7">
+        <v>171.98</v>
+      </c>
+      <c r="E7">
+        <v>239.88</v>
+      </c>
+      <c r="F7" s="17">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9">
+        <f>MEDIAN(B4:B7)</f>
+        <v>17.920000000000002</v>
+      </c>
+      <c r="C9">
+        <f>MEDIAN(C4:C7)</f>
+        <v>9.754999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13">
+        <f>Historicals!F11*$B$9</f>
+        <v>43884.646400000005</v>
+      </c>
+      <c r="C13">
+        <f>B13/Inputs!$B$22</f>
+        <v>431.18601328792676</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14">
+        <f>Historicals!F4*$C$9-Inputs!$B$19+Inputs!$B$21</f>
+        <v>34231.9715</v>
+      </c>
+      <c r="C14">
+        <f>B14/Inputs!$B$22</f>
+        <v>336.3442235248574</v>
       </c>
     </row>
   </sheetData>
@@ -1995,15 +3427,331 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8FB6CAA-755E-4048-8F46-C387A89B309E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.36328125" customWidth="1"/>
+    <col min="3" max="3" width="20.6328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>60</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G3" t="s">
+        <v>99</v>
+      </c>
+      <c r="H3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4">
+        <f>DCF!B20</f>
+        <v>479.55619117409594</v>
+      </c>
+      <c r="E4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F4" s="16">
+        <f>MIN(DCF!B29:F33)</f>
+        <v>345.95339591019837</v>
+      </c>
+      <c r="G4" s="16">
+        <f>MAX(DCF!B29:F33)</f>
+        <v>805.92849996945404</v>
+      </c>
+      <c r="H4" s="16">
+        <f>G4-F4</f>
+        <v>459.97510405925567</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="16">
+        <f>MIN(DCF!B29:F33)</f>
+        <v>345.95339591019837</v>
+      </c>
+      <c r="E5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F5">
+        <f>DCF!B20</f>
+        <v>479.55619117409594</v>
+      </c>
+      <c r="G5">
+        <f>DCF!B20</f>
+        <v>479.55619117409594</v>
+      </c>
+      <c r="H5">
+        <f>G5-F5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="16">
+        <f>MAX(DCF!B29:F33)</f>
+        <v>805.92849996945404</v>
+      </c>
+      <c r="E6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F6">
+        <f>Comps!C13</f>
+        <v>431.18601328792676</v>
+      </c>
+      <c r="G6">
+        <f>Comps!C13</f>
+        <v>431.18601328792676</v>
+      </c>
+      <c r="H6">
+        <f>G6-F6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7">
+        <f>Comps!C13</f>
+        <v>431.18601328792676</v>
+      </c>
+      <c r="E7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7">
+        <f>Comps!C14</f>
+        <v>336.3442235248574</v>
+      </c>
+      <c r="G7">
+        <f>Comps!C14</f>
+        <v>336.3442235248574</v>
+      </c>
+      <c r="H7">
+        <f>G7-F7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8">
+        <f>Comps!C14</f>
+        <v>336.3442235248574</v>
+      </c>
+      <c r="E8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F8">
+        <f>DCF!B22</f>
+        <v>1517.2</v>
+      </c>
+      <c r="G8">
+        <f>DCF!B22</f>
+        <v>1517.2</v>
+      </c>
+      <c r="H8">
+        <f>G8-F8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9">
+        <f>DCF!B22</f>
+        <v>1517.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="11">
+        <f>Inputs!B7</f>
+        <v>9.7485720303274723E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="13">
+        <f>Inputs!B8</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="11">
+        <f>Inputs!B2</f>
+        <v>0.1027756094442282</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="11">
+        <f>Inputs!B3</f>
+        <v>0.20889009323488397</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="11">
+        <f>Inputs!B4</f>
+        <v>0.25662000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="11">
+        <f>Inputs!B5</f>
+        <v>3.628E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" s="16">
+        <f>DCF!B16</f>
+        <v>48925.908646649492</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="16">
+        <f>DCF!B17</f>
+        <v>118.31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" s="16">
+        <f>DCF!B18</f>
+        <v>48807.598646649494</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="16">
+        <f>DCF!B19</f>
+        <v>101.7766</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="16">
+        <f>DCF!B20</f>
+        <v>479.55619117409594</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" s="15">
+        <f>DCF!B24</f>
+        <v>46290</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" s="16">
+        <f>Comps!B9</f>
+        <v>17.920000000000002</v>
+      </c>
+      <c r="C28" s="16">
+        <f>Comps!C13</f>
+        <v>431.18601328792676</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" s="16">
+        <f>Comps!C9</f>
+        <v>9.754999999999999</v>
+      </c>
+      <c r="C29" s="16">
+        <f>Comps!C14</f>
+        <v>336.3442235248574</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>